<commit_message>
Ajustar hiperparámetros en el modelo y optimización, modificar condiciones de filtrado en predicciones, y actualizar el número de pruebas en la optimización.
</commit_message>
<xml_diff>
--- a/mejores_hiperparametros.xlsx
+++ b/mejores_hiperparametros.xlsx
@@ -512,52 +512,60 @@
     </row>
     <row r="2">
       <c r="A2" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="B2" t="n">
-        <v>192</v>
+        <v>128</v>
       </c>
       <c r="C2" t="n">
-        <v>192</v>
+        <v>256</v>
       </c>
       <c r="D2" t="n">
-        <v>128</v>
+        <v>96</v>
       </c>
       <c r="E2" t="n">
-        <v>0.1669682694700993</v>
+        <v>0.4356815973587387</v>
       </c>
       <c r="F2" t="n">
-        <v>0.002990315296560121</v>
+        <v>0.007954866093105506</v>
       </c>
       <c r="G2" t="n">
-        <v>0.001076189765349653</v>
+        <v>0.0001086866899103121</v>
       </c>
       <c r="H2" t="n">
-        <v>384</v>
+        <v>256</v>
       </c>
       <c r="I2" t="n">
         <v>200</v>
       </c>
       <c r="J2" t="n">
-        <v>0.7309136390686035</v>
+        <v>0.2928660809993744</v>
       </c>
       <c r="K2" t="n">
-        <v>356.5070721333333</v>
+        <v>375.2114747833333</v>
       </c>
       <c r="L2" t="n">
-        <v>47</v>
-      </c>
-      <c r="M2" t="n">
-        <v>0.9584767818450928</v>
-      </c>
-      <c r="N2" t="n">
-        <v>0.6137502590815226</v>
-      </c>
-      <c r="O2" t="n">
-        <v>0.7309136390686035</v>
-      </c>
-      <c r="P2" t="n">
-        <v>1.530587951342265</v>
+        <v>61</v>
+      </c>
+      <c r="M2" t="inlineStr">
+        <is>
+          <t>[0.15247339010238647]</t>
+        </is>
+      </c>
+      <c r="N2" t="inlineStr">
+        <is>
+          <t>[4.093002796173096]</t>
+        </is>
+      </c>
+      <c r="O2" t="inlineStr">
+        <is>
+          <t>[0.2928660809993744]</t>
+        </is>
+      </c>
+      <c r="P2" t="inlineStr">
+        <is>
+          <t>[3.7240853309631348]</t>
+        </is>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
esta bien todos los cambios
</commit_message>
<xml_diff>
--- a/mejores_hiperparametros.xlsx
+++ b/mejores_hiperparametros.xlsx
@@ -512,25 +512,25 @@
     </row>
     <row r="2">
       <c r="A2" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="B2" t="n">
-        <v>128</v>
+        <v>384</v>
       </c>
       <c r="C2" t="n">
         <v>256</v>
       </c>
       <c r="D2" t="n">
-        <v>96</v>
+        <v>128</v>
       </c>
       <c r="E2" t="n">
-        <v>0.4356815973587387</v>
+        <v>0.3875188255460017</v>
       </c>
       <c r="F2" t="n">
-        <v>0.007954866093105506</v>
+        <v>0.008640737182527825</v>
       </c>
       <c r="G2" t="n">
-        <v>0.0001086866899103121</v>
+        <v>0.0001699336681260433</v>
       </c>
       <c r="H2" t="n">
         <v>256</v>
@@ -539,32 +539,32 @@
         <v>200</v>
       </c>
       <c r="J2" t="n">
-        <v>0.2928660809993744</v>
+        <v>0.5556946396827698</v>
       </c>
       <c r="K2" t="n">
-        <v>375.2114747833333</v>
+        <v>1057.943737616667</v>
       </c>
       <c r="L2" t="n">
-        <v>61</v>
+        <v>117</v>
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>[0.15247339010238647]</t>
+          <t>[0.3285311758518219]</t>
         </is>
       </c>
       <c r="N2" t="inlineStr">
         <is>
-          <t>[4.093002796173096]</t>
+          <t>[3.562859296798706]</t>
         </is>
       </c>
       <c r="O2" t="inlineStr">
         <is>
-          <t>[0.2928660809993744]</t>
+          <t>[0.5556946396827698]</t>
         </is>
       </c>
       <c r="P2" t="inlineStr">
         <is>
-          <t>[3.7240853309631348]</t>
+          <t>[3.0447330474853516]</t>
         </is>
       </c>
     </row>

</xml_diff>